<commit_message>
Add Balyasny + QRT to both sheets, fix row numbers
</commit_message>
<xml_diff>
--- a/New_Targets_US_HK_2026.xlsx
+++ b/New_Targets_US_HK_2026.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +100,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -479,7 +480,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Summer 2027 QR/QT Internships - New Targets (NOT yet applied, cross-checked vs 78 applied list) - compiled 2026-10-25</t>
+          <t>US Summer 2027 QR/QT Internships - New Targets (15 postings, cross-checked vs 78 applied) - compiled 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -720,6 +721,66 @@
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>https://quantroles.com/cities/new-york</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Balyasny Asset Management</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Quantitative Analyst - Commodities (Summer Internship, HK) + 11 NY internship roles incl. QR/Applied AI</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>New York / Hong Kong</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>https://quantroles.com/cities/new-york</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Qube Research &amp; Technologies (QRT)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>2027 Internship - Quantitative Research and Trading (+ FPGA/Data Eng/Infrastructure)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>New York / Hong Kong / Singapore</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>https://quantroles.com/cities/new-york</t>
         </is>
@@ -748,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -762,7 +823,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Hong Kong QR/QT Internships - New Targets (NOT yet applied, verified on quantroles.com) - compiled 2026-10-25</t>
+          <t>Hong Kong QR/QT Internships - New Targets (8 postings, verified on quantroles.com) - compiled 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -975,6 +1036,66 @@
       <c r="F9" s="8" t="inlineStr">
         <is>
           <t>https://campusjobs.mlp.com/careers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Balyasny Asset Management</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Quantitative Analyst - Commodities Investment Team (Summer Internship) + SWE Internship</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>https://quantroles.com/cities/hong-kong</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Qube Research &amp; Technologies (QRT)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>2027 Internship - Quantitative Research and Trading + Software Engineer and Quantitative Developer</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Hong Kong / Singapore</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>https://quantroles.com/cities/hong-kong</t>
         </is>
       </c>
     </row>

</xml_diff>